<commit_message>
Gate F F5.1: remediate implementation governance
</commit_message>
<xml_diff>
--- a/architecture/released/v1.11/RELEASE-MANIFEST-v1.11.xlsx
+++ b/architecture/released/v1.11/RELEASE-MANIFEST-v1.11.xlsx
@@ -419,7 +419,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H6" s="11" t="str">
-        <x:v>d4a0860c36933ea36777175c3fc3be98942346d485b3732f02570a88171f3a96</x:v>
+        <x:v>64845ff93ba869b1944d8e378238d17d76c3051c3a63cdb32d19c22eb1af02f1</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str">
         <x:v>ACR-001 v1.11</x:v>
@@ -483,7 +483,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H8" s="11" t="str">
-        <x:v>3c6c9340314e0035a760db795d7929cac4a5112ade79143835589cf9cb015af6</x:v>
+        <x:v>e5a652c2402433f78633a4c3461767bf79cc174d02dba90452ad3aa898d60a7d</x:v>
       </x:c>
       <x:c r="I8" s="11" t="str">
         <x:v/>
@@ -515,7 +515,7 @@
         <x:v>AUTHORITATIVE</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>eb115fe41338c9e75b518d116e076f56f853e90943fb1ba5ec326979ff6b4c45</x:v>
+        <x:v>e7049df863587420a0670d9025bf4526b733f03b32cc54e7a250750c61d742cd</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str">
         <x:v>Release README v1.10</x:v>

</xml_diff>